<commit_message>
Cập nhật Tuần 02: Thêm Slide bài giảng 9 lớp, cập nhật TKB Đậu Đình Nguyên, thêm Đơn xin nghỉ phép, xóa TKB GV cũ và scripts không dùng
</commit_message>
<xml_diff>
--- a/Thời khóa biểu giáo viên/Thời khóa biểu - Đậu Đình Nguyên.xlsx
+++ b/Thời khóa biểu giáo viên/Thời khóa biểu - Đậu Đình Nguyên.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TKB Cá Nhân" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TKB Đậu Đình Nguyên" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'TKB Đậu Đình Nguyên'!$A$1:$H$17</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,20 +30,63 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <sz val="13"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="15"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <i val="1"/>
+      <color rgb="001D2A64"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="00003C8C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="008C3C00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="001D2A64"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <i val="1"/>
+      <color rgb="00404060"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00003C8C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="008C3C00"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -50,18 +95,54 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="001D2A64"/>
+        <bgColor rgb="001D2A64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00253580"/>
+        <bgColor rgb="00253580"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF0FF"/>
+        <bgColor rgb="00EBF0FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4FF"/>
+        <bgColor rgb="00D6E4FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE5CC"/>
+        <bgColor rgb="00FFE5CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8ECF5"/>
+        <bgColor rgb="00E8ECF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FF"/>
+        <bgColor rgb="00F5F7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF3FF"/>
+        <bgColor rgb="00EFF3FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -71,44 +152,199 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00AAAACC"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00AAAACC"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00AAAACC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00AAAACC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001D2A64"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAACC"/>
+      </right>
+      <top style="medium">
+        <color rgb="001D2A64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAACC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAACC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAACC"/>
+      </right>
+      <top style="medium">
+        <color rgb="001D2A64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAACC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAACC"/>
+      </left>
+      <right style="medium">
+        <color rgb="001D2A64"/>
+      </right>
+      <top style="medium">
+        <color rgb="001D2A64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAACC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001D2A64"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAACC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAACC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAACC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAACC"/>
+      </left>
+      <right style="medium">
+        <color rgb="001D2A64"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAACC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAACC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001D2A64"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAACC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAACC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001D2A64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAACC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAACC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAACC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001D2A64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAACC"/>
+      </left>
+      <right style="medium">
+        <color rgb="001D2A64"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAACC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001D2A64"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,324 +710,468 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TRƯỜNG TIỂU HỌC VÀ THCS UNIGO</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>THỜI KHOÁ BIỂU CÁ NHÂN GIÁO VIÊN</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>THỜI KHOÁ BIỂU CÁ NHÂN GIÁO VIÊN  —  Năm học 2026–2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Giáo viên: Đậu Đình Nguyên | Bộ môn: Tin học &amp; Robotics | Tổng số: 25 tiết/tuần (Theo TKB toàn trường CHECK - chuẩn)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Buổi / Tiết</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+          <t>Giáo viên: Đậu Đình Nguyên   |   Bộ môn: Tin học &amp; Robotics   |   Tổng: 25 tiết/tuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>🔵 Xanh nhạt: Tin học</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>🟠 Cam nhạt: Robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Tiết</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Giờ TH</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Giờ THCS</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Thứ Hai</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Thứ Ba</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Thứ Tư</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Thứ Năm</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>Thứ Sáu</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>BUỔI SÁNG</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>▸   BUỔI SÁNG</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="11" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Tiết 1</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Tin (TT3)</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Tin (2C1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>8:15–8:50</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>8:05–8:50</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="n"/>
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(TT3)</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(2C1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Tiết 2</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (3A1)</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (1A1)</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (3C1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>8:55–9:30</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>8:55–9:40</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(3A1)</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(1A1)</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(3C1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Tiết 3</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Tin (5C1)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>9:45–10:20</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>9:45–10:25</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(5C1)</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="n"/>
+      <c r="G9" s="14" t="n"/>
+      <c r="H9" s="19" t="n"/>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Tiết 4</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Tin (1A1)</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (5C1)</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Tin (3C1)</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (2C1)</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Tin (6A1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>10:25–11:00</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>10:30–11:10</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(1A1)</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(5C1)</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(3C1)</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(2C1)</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(6A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Tiết 5</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (6A1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>BUỔI CHIỀU</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr"/>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>11:15–11:50</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
+      <c r="G11" s="14" t="n"/>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(6A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>▸   BUỔI CHIỀU</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Tiết 1</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Tin (2A1)</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Tin (3A1)</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Tin (8A1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>13:15–13:50</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>13:05–13:50</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(2A1)</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="n"/>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(3A1)</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(8A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Tiết 2</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Tin (1C1)</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Tin (TTH 1)</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (8A1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>13:55–14:30</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>13:55–14:40</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(1C1)</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="n"/>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(TTH 1)</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(8A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Tiết 3</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Tin (7A1)</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Tin (4C1)</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Tin (TTH2)</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (4C1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>14:55–15:30</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>14:50–15:30</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n"/>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(7A1)</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(4C1)</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(TTH2)</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(4C1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Tiết 4</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (7A1)</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (2A1)</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Robotics (1C1)</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>15:35–16:10</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>15:35–16:20</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(7A1)</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(2A1)</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(1C1)</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Tiết 5</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="8" t="n"/>
+      <c r="B17" s="21" t="inlineStr"/>
+      <c r="C17" s="21" t="inlineStr"/>
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="22" t="n"/>
+      <c r="F17" s="22" t="n"/>
+      <c r="G17" s="22" t="n"/>
+      <c r="H17" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A3:F3"/>
+  <mergeCells count="7">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A6:H6"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cập nhật Lịch báo giảng Tuần 30-35, slide bài giảng v3 Tin học (Tiền TH - Lớp 8) và các script hỗ trợ
</commit_message>
<xml_diff>
--- a/Thời khóa biểu giáo viên/Thời khóa biểu - Đậu Đình Nguyên.xlsx
+++ b/Thời khóa biểu giáo viên/Thời khóa biểu - Đậu Đình Nguyên.xlsx
@@ -323,16 +323,16 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -831,7 +831,12 @@
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
-      <c r="E7" s="14" t="n"/>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(1C1)</t>
+        </is>
+      </c>
       <c r="F7" s="14" t="n"/>
       <c r="G7" s="15" t="inlineStr">
         <is>
@@ -841,8 +846,8 @@
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>💻 Tin học
-(2C1)</t>
+          <t>🤖 Robotics
+(3C1)</t>
         </is>
       </c>
     </row>
@@ -876,12 +881,7 @@
 (1A1)</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>🤖 Robotics
-(3C1)</t>
-        </is>
-      </c>
+      <c r="H8" s="18" t="n"/>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="F9" s="14" t="n"/>
       <c r="G9" s="14" t="n"/>
-      <c r="H9" s="19" t="n"/>
+      <c r="H9" s="18" t="n"/>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
@@ -950,7 +950,7 @@
 (2C1)</t>
         </is>
       </c>
-      <c r="H10" s="16" t="inlineStr">
+      <c r="H10" s="19" t="inlineStr">
         <is>
           <t>💻 Tin học
 (6A1)</t>
@@ -973,7 +973,7 @@
       <c r="E11" s="14" t="n"/>
       <c r="F11" s="14" t="n"/>
       <c r="G11" s="14" t="n"/>
-      <c r="H11" s="18" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>🤖 Robotics
 (6A1)</t>
@@ -1024,7 +1024,7 @@
 (3A1)</t>
         </is>
       </c>
-      <c r="H13" s="16" t="inlineStr">
+      <c r="H13" s="19" t="inlineStr">
         <is>
           <t>💻 Tin học
 (8A1)</t>
@@ -1048,12 +1048,7 @@
         </is>
       </c>
       <c r="D14" s="14" t="n"/>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>💻 Tin học
-(1C1)</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="n"/>
       <c r="F14" s="14" t="n"/>
       <c r="G14" s="15" t="inlineStr">
         <is>
@@ -1061,7 +1056,7 @@
 (TTH 1)</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>🤖 Robotics
 (8A1)</t>
@@ -1084,7 +1079,12 @@
           <t>14:50–15:30</t>
         </is>
       </c>
-      <c r="D15" s="14" t="n"/>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>💻 Tin học
+(2C1)</t>
+        </is>
+      </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
           <t>💻 Tin học
@@ -1103,7 +1103,7 @@
 (TTH2)</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>🤖 Robotics
 (4C1)</t>
@@ -1145,7 +1145,7 @@
 (1C1)</t>
         </is>
       </c>
-      <c r="H16" s="19" t="n"/>
+      <c r="H16" s="18" t="n"/>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="20" t="inlineStr">

</xml_diff>